<commit_message>
Ver2.09 Add zoom,w,h on canva 03
</commit_message>
<xml_diff>
--- a/public/config/default.xlsx
+++ b/public/config/default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IKEGAMI\JAVAscript\SerialRecoder\serial-app\public\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F81BF7C-242E-4F60-900F-04ADF033ED40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A9D037-E800-40B1-B33E-AC57A4E596D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="62100" yWindow="2895" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="25">
   <si>
     <t>Model</t>
     <phoneticPr fontId="1"/>
@@ -83,6 +83,37 @@
   <si>
     <t>Value</t>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>PS1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>PS2</t>
+  </si>
+  <si>
+    <t>PS3</t>
+  </si>
+  <si>
+    <t>PS4</t>
+  </si>
+  <si>
+    <t>PS5</t>
+  </si>
+  <si>
+    <t>PS6</t>
+  </si>
+  <si>
+    <t>PS7</t>
+  </si>
+  <si>
+    <t>PS8</t>
+  </si>
+  <si>
+    <t>Export Time</t>
+  </si>
+  <si>
+    <t>2026/9/30 9:38:24</t>
   </si>
 </sst>
 </file>
@@ -416,15 +447,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A2:C21"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="11.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
@@ -440,15 +475,18 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>12</v>
@@ -456,23 +494,23 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>12</v>
@@ -480,25 +518,97 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B13" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
loard exprt format change
</commit_message>
<xml_diff>
--- a/public/config/default.xlsx
+++ b/public/config/default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IKEGAMI\JAVAscript\SerialRecoder\serial-app\public\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A69F19-C0A5-4989-AAAF-85D43A9CF445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92600508-93B6-463A-A3D2-FD4AE27BC200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="59970" yWindow="1770" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57495" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -502,8 +502,8 @@
   <cols>
     <col min="1" max="1" width="11.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="46.625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.4">
@@ -514,10 +514,10 @@
         <v>3</v>
       </c>
       <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
         <v>14</v>
-      </c>
-      <c r="D1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
@@ -525,7 +525,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="1"/>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -533,7 +533,7 @@
       <c r="A3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>24</v>
       </c>
     </row>
@@ -542,7 +542,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="1"/>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>1</v>
       </c>
     </row>
@@ -569,7 +569,7 @@
       <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D7" t="s">
+      <c r="C7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -580,7 +580,7 @@
       <c r="B8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D8" t="s">
+      <c r="C8" t="s">
         <v>29</v>
       </c>
     </row>
@@ -591,7 +591,7 @@
       <c r="B9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D9" t="s">
+      <c r="C9" t="s">
         <v>30</v>
       </c>
     </row>
@@ -686,7 +686,7 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{D9E34957-D486-4A13-9044-4494FDBFBD22}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{D9E34957-D486-4A13-9044-4494FDBFBD22}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>